<commit_message>
Added the battery regulation (not ingested yet) and added loading plus more accessible user input
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/isabel_rutten_tno_nl/Documents/GitHub/dpp-docs-preprocessing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/isabel_rutten_tno_nl/Documents/GitHub/diff/system-ai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="552" documentId="11_F25DC773A252ABDACC10485FE99F4AEE5ADE58F4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0C84293-7560-4B6D-97A0-4A2F11A4045E}"/>
+  <xr:revisionPtr revIDLastSave="565" documentId="11_F25DC773A252ABDACC10485FE99F4AEE5ADE58F4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC77092-86EF-40C0-98C3-EFBA6AD40B50}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="207">
   <si>
     <t>ID</t>
   </si>
@@ -654,6 +654,16 @@
   </si>
   <si>
     <t>Regulation (EU) 2024/3015 lays down rules prohibiting economic operators1 from placing and making available on the European Union (EU) market, or exporting from it, products made with forced labour2, to improve the functioning of the internal market and contribute to the fight against forced labour.</t>
+  </si>
+  <si>
+    <t>di-09</t>
+  </si>
+  <si>
+    <t>Regulation (EU) 2023/1542 of the European Parliament and of the Council of 12 July 2023 concerning batteries and waste batteries, amending Directive 2008/98/EC and Regulation (EU) 2019/1020 and repealing Directive 2006/66/EC (Text with EEA relevance)</t>
+  </si>
+  <si>
+    <t>Regulation (EU) 2023/1542 aims to ensure that, in the future, batteries have a low carbon footprint, use minimal harmful substances, need fewer raw materials from non-European Union (EU) countries and are collected, reused and recycled to a high degree within the EU.
+The regulation is part of the EU’s shift towards a circular economy, an important aspect of the European Green Deal (see summary), and will increase security of supply for raw materials and energy, along with enhancing the EU’s strategic autonomy and competitiveness.</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA8CC663-10E6-4434-B845-7C0EC55EC8D7}">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" customWidth="1"/>
@@ -2210,6 +2220,35 @@
       </c>
       <c r="I41" s="1">
         <v>47384</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>204</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="1">
+        <v>45340</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F42" t="s">
+        <v>157</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="H42" t="s">
+        <v>141</v>
+      </c>
+      <c r="I42" s="1">
+        <v>46436</v>
       </c>
     </row>
   </sheetData>
@@ -2248,6 +2287,7 @@
     <hyperlink ref="E39" r:id="rId31" xr:uid="{E5AE9862-37C5-49F2-8AA6-F4C302DD8CBF}"/>
     <hyperlink ref="E40" r:id="rId32" xr:uid="{A71BC7BF-9FA1-4643-A147-F4B8DB719351}"/>
     <hyperlink ref="E41" r:id="rId33" xr:uid="{083DD598-9B70-447A-9D44-13FCD40BBF9B}"/>
+    <hyperlink ref="E42" r:id="rId34" xr:uid="{EC32493B-3320-48F2-88F8-9858176F1B2B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>